<commit_message>
added up do date documents for week 3
</commit_message>
<xml_diff>
--- a/4_Language/SW3_Project Management/ET-PM3_SW3_Project Management-GanttChart-Template.xlsx
+++ b/4_Language/SW3_Project Management/ET-PM3_SW3_Project Management-GanttChart-Template.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29227"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F30FA55-09AF-43B4-87B6-BEA6DF7D0E84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{443A09F0-E9F8-F745-967E-695C0F4F8E7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="11280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3400" yWindow="2480" windowWidth="29660" windowHeight="17680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ProjectSchedule" sheetId="11" r:id="rId1"/>
@@ -20,7 +20,7 @@
     <definedName name="task_start" localSheetId="0">ProjectSchedule!$E1</definedName>
     <definedName name="today" localSheetId="0">TODAY()</definedName>
   </definedNames>
-  <calcPr calcId="191028" iterateDelta="1E-4"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="167" uniqueCount="58">
   <si>
     <t>Create a Project Schedule in this worksheet.
 Enter title of this project in cell B1. 
@@ -53,6 +53,9 @@
   </si>
   <si>
     <t>Enter Company Name in cell B2.</t>
+  </si>
+  <si>
+    <t>GROUP</t>
   </si>
   <si>
     <t>Enter the name of the Project Lead in cell B3. Enter the Project Start date in cell E3. Pooject Start: label is in cell C3.</t>
@@ -127,6 +130,9 @@
 To delete the phase and work only from tasks, simply delete this row.</t>
   </si>
   <si>
+    <t>Phase 1 Title</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cell B9 contains the sample task "Task 1." 
 Enter a new task name in cell B9.
 Enter a person to assign the task to in cell C9.
@@ -136,10 +142,19 @@
 A status bar shaded for the dates entered appears in blocks starting from cell I9 through BL9. </t>
   </si>
   <si>
+    <t>Time planned</t>
+  </si>
+  <si>
+    <t>Name</t>
+  </si>
+  <si>
     <t>Rows 10 through 13 repeat the pattern from row 9. 
 Repeat the instructions from cell A9 for all task rows in this worksheet. Overwrite any sample data.
 A sample of another phase starts in cell A14. 
 Continue entering tasks in cells A10 through A13 or go to cell A14 to learn more.</t>
+  </si>
+  <si>
+    <t>Time used</t>
   </si>
   <si>
     <t>Task 3</t>
@@ -161,6 +176,9 @@
 Repeat the instructions from cells A8 and A9 whenever you need to.</t>
   </si>
   <si>
+    <t>Phase 2 Title</t>
+  </si>
+  <si>
     <t>Task 1</t>
   </si>
   <si>
@@ -237,48 +255,6 @@
   </si>
   <si>
     <t>Businesses will find invoices, time sheets, inventory trackers, financial statements, and project planning templates. Teachers and students will find resources such as class schedules, grade books, and attendance sheets. Organize your family life with meal planners, checklists, and exercise logs. Each template is thoroughly researched, refined, and improved over time through feedback from thousands of users.</t>
-  </si>
-  <si>
-    <t>Phase 1: HW Development</t>
-  </si>
-  <si>
-    <t>PCB Layout</t>
-  </si>
-  <si>
-    <t>LTspice Simulation</t>
-  </si>
-  <si>
-    <t>Assembly</t>
-  </si>
-  <si>
-    <t>Schematic Design</t>
-  </si>
-  <si>
-    <t>HW Report</t>
-  </si>
-  <si>
-    <t>HW Demo</t>
-  </si>
-  <si>
-    <t>Testing (+ Report)</t>
-  </si>
-  <si>
-    <t>Thomas, Bogdan</t>
-  </si>
-  <si>
-    <t>Bogdan</t>
-  </si>
-  <si>
-    <t>Thomas</t>
-  </si>
-  <si>
-    <t>Submit HW Report</t>
-  </si>
-  <si>
-    <t>Phase 2: FW Development</t>
-  </si>
-  <si>
-    <t>Thomas Perri &amp; Bogdans Grebnevs</t>
   </si>
 </sst>
 </file>
@@ -293,7 +269,7 @@
     <numFmt numFmtId="168" formatCode="d"/>
     <numFmt numFmtId="169" formatCode="yyyy\-mm\-dd;@"/>
   </numFmts>
-  <fonts count="24" x14ac:knownFonts="1">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -454,13 +430,6 @@
     <font>
       <sz val="11"/>
       <color theme="0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -697,7 +666,7 @@
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="95">
+  <cellXfs count="92">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -939,15 +908,6 @@
     <xf numFmtId="169" fontId="9" fillId="4" borderId="2" xfId="10" applyNumberFormat="1" applyFill="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="169" fontId="23" fillId="3" borderId="2" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="3" borderId="2" xfId="12" applyFont="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="169" fontId="5" fillId="3" borderId="2" xfId="10" applyNumberFormat="1" applyFont="1" applyFill="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="167" fontId="0" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
@@ -957,16 +917,16 @@
     <xf numFmtId="167" fontId="0" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="14" fontId="9" fillId="0" borderId="3" xfId="9" applyNumberFormat="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="8" applyAlignment="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="8" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" indent="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="3" xfId="9" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="8">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="8" applyBorder="1">
-      <alignment horizontal="right" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="13">
     <cellStyle name="Comma" xfId="4" builtinId="3" customBuiltin="1"/>
@@ -1545,21 +1505,21 @@
   <sheetPr codeName="Sheet1">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:CU39"/>
-  <sheetFormatPr defaultColWidth="8.7265625" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:CU36"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="30" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="2.7265625" style="58" customWidth="1"/>
-    <col min="2" max="2" width="19.81640625" customWidth="1"/>
-    <col min="3" max="3" width="30.7265625" customWidth="1"/>
-    <col min="4" max="4" width="10.7265625" customWidth="1"/>
-    <col min="5" max="5" width="10.453125" style="5" customWidth="1"/>
-    <col min="6" max="6" width="10.453125" customWidth="1"/>
-    <col min="7" max="7" width="2.7265625" customWidth="1"/>
-    <col min="8" max="8" width="6.1796875" customWidth="1"/>
-    <col min="9" max="99" width="2.453125" customWidth="1"/>
+    <col min="1" max="1" width="2.7109375" style="58" customWidth="1"/>
+    <col min="2" max="2" width="19.85546875" customWidth="1"/>
+    <col min="3" max="3" width="30.7109375" customWidth="1"/>
+    <col min="4" max="4" width="10.7109375" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" style="5" customWidth="1"/>
+    <col min="6" max="6" width="10.42578125" customWidth="1"/>
+    <col min="7" max="7" width="2.7109375" customWidth="1"/>
+    <col min="8" max="8" width="6.140625" customWidth="1"/>
+    <col min="9" max="99" width="2.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:99" ht="30" customHeight="1" x14ac:dyDescent="0.65">
+    <row r="1" spans="1:99" ht="30" customHeight="1">
       <c r="A1" s="59" t="s">
         <v>0</v>
       </c>
@@ -1573,851 +1533,852 @@
       <c r="H1" s="2"/>
       <c r="I1" s="14"/>
     </row>
-    <row r="2" spans="1:99" ht="30" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:99" ht="30" customHeight="1">
       <c r="A2" s="58" t="s">
         <v>2</v>
       </c>
       <c r="B2" s="64" t="s">
-        <v>65</v>
+        <v>3</v>
       </c>
       <c r="I2" s="61"/>
     </row>
-    <row r="3" spans="1:99" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:99" ht="30" customHeight="1">
       <c r="A3" s="58" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B3" s="65"/>
-      <c r="C3" s="92" t="s">
-        <v>4</v>
-      </c>
-      <c r="D3" s="93"/>
-      <c r="E3" s="91">
-        <v>45919</v>
-      </c>
-      <c r="F3" s="91"/>
+      <c r="C3" s="88" t="s">
+        <v>5</v>
+      </c>
+      <c r="D3" s="89"/>
+      <c r="E3" s="90">
+        <f ca="1">TODAY()</f>
+        <v>45909</v>
+      </c>
+      <c r="F3" s="90"/>
     </row>
-    <row r="4" spans="1:99" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:99" ht="30" customHeight="1">
       <c r="A4" s="59" t="s">
-        <v>5</v>
-      </c>
-      <c r="C4" s="92" t="s">
         <v>6</v>
       </c>
-      <c r="D4" s="93"/>
+      <c r="C4" s="88" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="89"/>
       <c r="E4" s="7">
         <v>1</v>
       </c>
-      <c r="I4" s="88">
-        <f>M5</f>
+      <c r="I4" s="85">
+        <f ca="1">I5</f>
+        <v>45908</v>
+      </c>
+      <c r="J4" s="86"/>
+      <c r="K4" s="86"/>
+      <c r="L4" s="86"/>
+      <c r="M4" s="86"/>
+      <c r="N4" s="86"/>
+      <c r="O4" s="87"/>
+      <c r="P4" s="85">
+        <f ca="1">M5</f>
+        <v>45912</v>
+      </c>
+      <c r="Q4" s="86"/>
+      <c r="R4" s="86"/>
+      <c r="S4" s="86"/>
+      <c r="T4" s="86"/>
+      <c r="U4" s="86"/>
+      <c r="V4" s="87"/>
+      <c r="W4" s="85">
+        <f ca="1">W5</f>
+        <v>45922</v>
+      </c>
+      <c r="X4" s="86"/>
+      <c r="Y4" s="86"/>
+      <c r="Z4" s="86"/>
+      <c r="AA4" s="86"/>
+      <c r="AB4" s="86"/>
+      <c r="AC4" s="87"/>
+      <c r="AD4" s="85">
+        <f ca="1">AD5</f>
+        <v>45929</v>
+      </c>
+      <c r="AE4" s="86"/>
+      <c r="AF4" s="86"/>
+      <c r="AG4" s="86"/>
+      <c r="AH4" s="86"/>
+      <c r="AI4" s="86"/>
+      <c r="AJ4" s="87"/>
+      <c r="AK4" s="85">
+        <f ca="1">AK5</f>
+        <v>45936</v>
+      </c>
+      <c r="AL4" s="86"/>
+      <c r="AM4" s="86"/>
+      <c r="AN4" s="86"/>
+      <c r="AO4" s="86"/>
+      <c r="AP4" s="86"/>
+      <c r="AQ4" s="87"/>
+      <c r="AR4" s="85">
+        <f ca="1">AR5</f>
+        <v>45943</v>
+      </c>
+      <c r="AS4" s="86"/>
+      <c r="AT4" s="86"/>
+      <c r="AU4" s="86"/>
+      <c r="AV4" s="86"/>
+      <c r="AW4" s="86"/>
+      <c r="AX4" s="87"/>
+      <c r="AY4" s="85">
+        <f ca="1">AY5</f>
+        <v>45950</v>
+      </c>
+      <c r="AZ4" s="86"/>
+      <c r="BA4" s="86"/>
+      <c r="BB4" s="86"/>
+      <c r="BC4" s="86"/>
+      <c r="BD4" s="86"/>
+      <c r="BE4" s="87"/>
+      <c r="BF4" s="85">
+        <f ca="1">BF5</f>
+        <v>45957</v>
+      </c>
+      <c r="BG4" s="86"/>
+      <c r="BH4" s="86"/>
+      <c r="BI4" s="86"/>
+      <c r="BJ4" s="86"/>
+      <c r="BK4" s="86"/>
+      <c r="BL4" s="87"/>
+      <c r="BM4" s="85">
+        <f ca="1">BM5</f>
+        <v>45964</v>
+      </c>
+      <c r="BN4" s="86"/>
+      <c r="BO4" s="86"/>
+      <c r="BP4" s="86"/>
+      <c r="BQ4" s="86"/>
+      <c r="BR4" s="86"/>
+      <c r="BS4" s="87"/>
+      <c r="BT4" s="85">
+        <f ca="1">BT5</f>
+        <v>45971</v>
+      </c>
+      <c r="BU4" s="86"/>
+      <c r="BV4" s="86"/>
+      <c r="BW4" s="86"/>
+      <c r="BX4" s="86"/>
+      <c r="BY4" s="86"/>
+      <c r="BZ4" s="87"/>
+      <c r="CA4" s="85">
+        <f ca="1">CA5</f>
+        <v>45978</v>
+      </c>
+      <c r="CB4" s="86"/>
+      <c r="CC4" s="86"/>
+      <c r="CD4" s="86"/>
+      <c r="CE4" s="86"/>
+      <c r="CF4" s="86"/>
+      <c r="CG4" s="87"/>
+      <c r="CH4" s="85">
+        <f ca="1">CH5</f>
+        <v>45985</v>
+      </c>
+      <c r="CI4" s="86"/>
+      <c r="CJ4" s="86"/>
+      <c r="CK4" s="86"/>
+      <c r="CL4" s="86"/>
+      <c r="CM4" s="86"/>
+      <c r="CN4" s="87"/>
+      <c r="CO4" s="85">
+        <f ca="1">CO5</f>
+        <v>45992</v>
+      </c>
+      <c r="CP4" s="86"/>
+      <c r="CQ4" s="86"/>
+      <c r="CR4" s="86"/>
+      <c r="CS4" s="86"/>
+      <c r="CT4" s="86"/>
+      <c r="CU4" s="87"/>
+    </row>
+    <row r="5" spans="1:99" ht="15" customHeight="1">
+      <c r="A5" s="59" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="91"/>
+      <c r="C5" s="91"/>
+      <c r="D5" s="91"/>
+      <c r="E5" s="91"/>
+      <c r="F5" s="91"/>
+      <c r="G5" s="91"/>
+      <c r="I5" s="11">
+        <f ca="1">Project_Start-WEEKDAY(Project_Start,1)+2+7*(Display_Week-1)</f>
+        <v>45908</v>
+      </c>
+      <c r="J5" s="10">
+        <f ca="1">I5+1</f>
+        <v>45909</v>
+      </c>
+      <c r="K5" s="10">
+        <f t="shared" ref="K5:AX5" ca="1" si="0">J5+1</f>
+        <v>45910</v>
+      </c>
+      <c r="L5" s="10">
+        <f t="shared" ca="1" si="0"/>
+        <v>45911</v>
+      </c>
+      <c r="M5" s="10">
+        <f t="shared" ca="1" si="0"/>
+        <v>45912</v>
+      </c>
+      <c r="N5" s="10">
+        <f t="shared" ca="1" si="0"/>
+        <v>45913</v>
+      </c>
+      <c r="O5" s="12">
+        <f t="shared" ca="1" si="0"/>
+        <v>45914</v>
+      </c>
+      <c r="P5" s="11">
+        <f ca="1">O5+1</f>
+        <v>45915</v>
+      </c>
+      <c r="Q5" s="10">
+        <f ca="1">P5+1</f>
+        <v>45916</v>
+      </c>
+      <c r="R5" s="10">
+        <f t="shared" ca="1" si="0"/>
+        <v>45917</v>
+      </c>
+      <c r="S5" s="10">
+        <f t="shared" ca="1" si="0"/>
+        <v>45918</v>
+      </c>
+      <c r="T5" s="10">
+        <f t="shared" ca="1" si="0"/>
         <v>45919</v>
       </c>
-      <c r="J4" s="89"/>
-      <c r="K4" s="89"/>
-      <c r="L4" s="89"/>
-      <c r="M4" s="89"/>
-      <c r="N4" s="89"/>
-      <c r="O4" s="90"/>
-      <c r="P4" s="88">
-        <f>T5</f>
+      <c r="U5" s="10">
+        <f t="shared" ca="1" si="0"/>
+        <v>45920</v>
+      </c>
+      <c r="V5" s="12">
+        <f t="shared" ca="1" si="0"/>
+        <v>45921</v>
+      </c>
+      <c r="W5" s="11">
+        <f ca="1">V5+1</f>
+        <v>45922</v>
+      </c>
+      <c r="X5" s="10">
+        <f ca="1">W5+1</f>
+        <v>45923</v>
+      </c>
+      <c r="Y5" s="10">
+        <f t="shared" ca="1" si="0"/>
+        <v>45924</v>
+      </c>
+      <c r="Z5" s="10">
+        <f t="shared" ca="1" si="0"/>
+        <v>45925</v>
+      </c>
+      <c r="AA5" s="10">
+        <f t="shared" ca="1" si="0"/>
         <v>45926</v>
       </c>
-      <c r="Q4" s="89"/>
-      <c r="R4" s="89"/>
-      <c r="S4" s="89"/>
-      <c r="T4" s="89"/>
-      <c r="U4" s="89"/>
-      <c r="V4" s="90"/>
-      <c r="W4" s="88">
-        <f t="shared" ref="W4" si="0">AA5</f>
+      <c r="AB5" s="10">
+        <f t="shared" ca="1" si="0"/>
+        <v>45927</v>
+      </c>
+      <c r="AC5" s="12">
+        <f t="shared" ca="1" si="0"/>
+        <v>45928</v>
+      </c>
+      <c r="AD5" s="11">
+        <f ca="1">AC5+1</f>
+        <v>45929</v>
+      </c>
+      <c r="AE5" s="10">
+        <f ca="1">AD5+1</f>
+        <v>45930</v>
+      </c>
+      <c r="AF5" s="10">
+        <f t="shared" ca="1" si="0"/>
+        <v>45931</v>
+      </c>
+      <c r="AG5" s="10">
+        <f t="shared" ca="1" si="0"/>
+        <v>45932</v>
+      </c>
+      <c r="AH5" s="10">
+        <f t="shared" ca="1" si="0"/>
         <v>45933</v>
       </c>
-      <c r="X4" s="89"/>
-      <c r="Y4" s="89"/>
-      <c r="Z4" s="89"/>
-      <c r="AA4" s="89"/>
-      <c r="AB4" s="89"/>
-      <c r="AC4" s="90"/>
-      <c r="AD4" s="88">
-        <f t="shared" ref="AD4" si="1">AH5</f>
+      <c r="AI5" s="10">
+        <f t="shared" ca="1" si="0"/>
+        <v>45934</v>
+      </c>
+      <c r="AJ5" s="12">
+        <f t="shared" ca="1" si="0"/>
+        <v>45935</v>
+      </c>
+      <c r="AK5" s="11">
+        <f ca="1">AJ5+1</f>
+        <v>45936</v>
+      </c>
+      <c r="AL5" s="10">
+        <f ca="1">AK5+1</f>
+        <v>45937</v>
+      </c>
+      <c r="AM5" s="10">
+        <f t="shared" ca="1" si="0"/>
+        <v>45938</v>
+      </c>
+      <c r="AN5" s="10">
+        <f t="shared" ca="1" si="0"/>
+        <v>45939</v>
+      </c>
+      <c r="AO5" s="10">
+        <f t="shared" ca="1" si="0"/>
         <v>45940</v>
       </c>
-      <c r="AE4" s="89"/>
-      <c r="AF4" s="89"/>
-      <c r="AG4" s="89"/>
-      <c r="AH4" s="89"/>
-      <c r="AI4" s="89"/>
-      <c r="AJ4" s="90"/>
-      <c r="AK4" s="88">
-        <f t="shared" ref="AK4" si="2">AO5</f>
+      <c r="AP5" s="10">
+        <f t="shared" ca="1" si="0"/>
+        <v>45941</v>
+      </c>
+      <c r="AQ5" s="12">
+        <f t="shared" ca="1" si="0"/>
+        <v>45942</v>
+      </c>
+      <c r="AR5" s="11">
+        <f ca="1">AQ5+1</f>
+        <v>45943</v>
+      </c>
+      <c r="AS5" s="10">
+        <f ca="1">AR5+1</f>
+        <v>45944</v>
+      </c>
+      <c r="AT5" s="10">
+        <f t="shared" ca="1" si="0"/>
+        <v>45945</v>
+      </c>
+      <c r="AU5" s="10">
+        <f t="shared" ca="1" si="0"/>
+        <v>45946</v>
+      </c>
+      <c r="AV5" s="10">
+        <f t="shared" ca="1" si="0"/>
         <v>45947</v>
       </c>
-      <c r="AL4" s="89"/>
-      <c r="AM4" s="89"/>
-      <c r="AN4" s="89"/>
-      <c r="AO4" s="89"/>
-      <c r="AP4" s="89"/>
-      <c r="AQ4" s="90"/>
-      <c r="AR4" s="88">
-        <f t="shared" ref="AR4" si="3">AV5</f>
+      <c r="AW5" s="10">
+        <f t="shared" ca="1" si="0"/>
+        <v>45948</v>
+      </c>
+      <c r="AX5" s="12">
+        <f t="shared" ca="1" si="0"/>
+        <v>45949</v>
+      </c>
+      <c r="AY5" s="11">
+        <f ca="1">AX5+1</f>
+        <v>45950</v>
+      </c>
+      <c r="AZ5" s="10">
+        <f ca="1">AY5+1</f>
+        <v>45951</v>
+      </c>
+      <c r="BA5" s="10">
+        <f t="shared" ref="BA5:BE5" ca="1" si="1">AZ5+1</f>
+        <v>45952</v>
+      </c>
+      <c r="BB5" s="10">
+        <f t="shared" ca="1" si="1"/>
+        <v>45953</v>
+      </c>
+      <c r="BC5" s="10">
+        <f t="shared" ca="1" si="1"/>
         <v>45954</v>
       </c>
-      <c r="AS4" s="89"/>
-      <c r="AT4" s="89"/>
-      <c r="AU4" s="89"/>
-      <c r="AV4" s="89"/>
-      <c r="AW4" s="89"/>
-      <c r="AX4" s="90"/>
-      <c r="AY4" s="88">
-        <f t="shared" ref="AY4" si="4">BC5</f>
+      <c r="BD5" s="10">
+        <f t="shared" ca="1" si="1"/>
+        <v>45955</v>
+      </c>
+      <c r="BE5" s="12">
+        <f t="shared" ca="1" si="1"/>
+        <v>45956</v>
+      </c>
+      <c r="BF5" s="11">
+        <f ca="1">BE5+1</f>
+        <v>45957</v>
+      </c>
+      <c r="BG5" s="10">
+        <f ca="1">BF5+1</f>
+        <v>45958</v>
+      </c>
+      <c r="BH5" s="10">
+        <f t="shared" ref="BH5:BL5" ca="1" si="2">BG5+1</f>
+        <v>45959</v>
+      </c>
+      <c r="BI5" s="10">
+        <f t="shared" ca="1" si="2"/>
+        <v>45960</v>
+      </c>
+      <c r="BJ5" s="10">
+        <f t="shared" ca="1" si="2"/>
         <v>45961</v>
       </c>
-      <c r="AZ4" s="89"/>
-      <c r="BA4" s="89"/>
-      <c r="BB4" s="89"/>
-      <c r="BC4" s="89"/>
-      <c r="BD4" s="89"/>
-      <c r="BE4" s="90"/>
-      <c r="BF4" s="88">
-        <f t="shared" ref="BF4" si="5">BJ5</f>
+      <c r="BK5" s="10">
+        <f t="shared" ca="1" si="2"/>
+        <v>45962</v>
+      </c>
+      <c r="BL5" s="12">
+        <f t="shared" ca="1" si="2"/>
+        <v>45963</v>
+      </c>
+      <c r="BM5" s="12">
+        <f t="shared" ref="BM5" ca="1" si="3">BL5+1</f>
+        <v>45964</v>
+      </c>
+      <c r="BN5" s="12">
+        <f t="shared" ref="BN5" ca="1" si="4">BM5+1</f>
+        <v>45965</v>
+      </c>
+      <c r="BO5" s="12">
+        <f t="shared" ref="BO5" ca="1" si="5">BN5+1</f>
+        <v>45966</v>
+      </c>
+      <c r="BP5" s="12">
+        <f t="shared" ref="BP5" ca="1" si="6">BO5+1</f>
+        <v>45967</v>
+      </c>
+      <c r="BQ5" s="12">
+        <f t="shared" ref="BQ5" ca="1" si="7">BP5+1</f>
         <v>45968</v>
       </c>
-      <c r="BG4" s="89"/>
-      <c r="BH4" s="89"/>
-      <c r="BI4" s="89"/>
-      <c r="BJ4" s="89"/>
-      <c r="BK4" s="89"/>
-      <c r="BL4" s="90"/>
-      <c r="BM4" s="88">
-        <f t="shared" ref="BM4" si="6">BQ5</f>
+      <c r="BR5" s="12">
+        <f t="shared" ref="BR5" ca="1" si="8">BQ5+1</f>
+        <v>45969</v>
+      </c>
+      <c r="BS5" s="12">
+        <f t="shared" ref="BS5" ca="1" si="9">BR5+1</f>
+        <v>45970</v>
+      </c>
+      <c r="BT5" s="12">
+        <f t="shared" ref="BT5" ca="1" si="10">BS5+1</f>
+        <v>45971</v>
+      </c>
+      <c r="BU5" s="12">
+        <f t="shared" ref="BU5" ca="1" si="11">BT5+1</f>
+        <v>45972</v>
+      </c>
+      <c r="BV5" s="12">
+        <f t="shared" ref="BV5" ca="1" si="12">BU5+1</f>
+        <v>45973</v>
+      </c>
+      <c r="BW5" s="12">
+        <f t="shared" ref="BW5" ca="1" si="13">BV5+1</f>
+        <v>45974</v>
+      </c>
+      <c r="BX5" s="12">
+        <f t="shared" ref="BX5" ca="1" si="14">BW5+1</f>
         <v>45975</v>
       </c>
-      <c r="BN4" s="89"/>
-      <c r="BO4" s="89"/>
-      <c r="BP4" s="89"/>
-      <c r="BQ4" s="89"/>
-      <c r="BR4" s="89"/>
-      <c r="BS4" s="90"/>
-      <c r="BT4" s="88">
-        <f t="shared" ref="BT4" si="7">BX5</f>
+      <c r="BY5" s="12">
+        <f t="shared" ref="BY5" ca="1" si="15">BX5+1</f>
+        <v>45976</v>
+      </c>
+      <c r="BZ5" s="12">
+        <f t="shared" ref="BZ5" ca="1" si="16">BY5+1</f>
+        <v>45977</v>
+      </c>
+      <c r="CA5" s="12">
+        <f t="shared" ref="CA5" ca="1" si="17">BZ5+1</f>
+        <v>45978</v>
+      </c>
+      <c r="CB5" s="12">
+        <f t="shared" ref="CB5" ca="1" si="18">CA5+1</f>
+        <v>45979</v>
+      </c>
+      <c r="CC5" s="12">
+        <f t="shared" ref="CC5" ca="1" si="19">CB5+1</f>
+        <v>45980</v>
+      </c>
+      <c r="CD5" s="12">
+        <f t="shared" ref="CD5" ca="1" si="20">CC5+1</f>
+        <v>45981</v>
+      </c>
+      <c r="CE5" s="12">
+        <f t="shared" ref="CE5" ca="1" si="21">CD5+1</f>
         <v>45982</v>
       </c>
-      <c r="BU4" s="89"/>
-      <c r="BV4" s="89"/>
-      <c r="BW4" s="89"/>
-      <c r="BX4" s="89"/>
-      <c r="BY4" s="89"/>
-      <c r="BZ4" s="90"/>
-      <c r="CA4" s="88">
-        <f t="shared" ref="CA4" si="8">CE5</f>
+      <c r="CF5" s="12">
+        <f t="shared" ref="CF5" ca="1" si="22">CE5+1</f>
+        <v>45983</v>
+      </c>
+      <c r="CG5" s="12">
+        <f t="shared" ref="CG5" ca="1" si="23">CF5+1</f>
+        <v>45984</v>
+      </c>
+      <c r="CH5" s="12">
+        <f t="shared" ref="CH5" ca="1" si="24">CG5+1</f>
+        <v>45985</v>
+      </c>
+      <c r="CI5" s="12">
+        <f t="shared" ref="CI5" ca="1" si="25">CH5+1</f>
+        <v>45986</v>
+      </c>
+      <c r="CJ5" s="12">
+        <f t="shared" ref="CJ5" ca="1" si="26">CI5+1</f>
+        <v>45987</v>
+      </c>
+      <c r="CK5" s="12">
+        <f t="shared" ref="CK5" ca="1" si="27">CJ5+1</f>
+        <v>45988</v>
+      </c>
+      <c r="CL5" s="12">
+        <f t="shared" ref="CL5" ca="1" si="28">CK5+1</f>
         <v>45989</v>
       </c>
-      <c r="CB4" s="89"/>
-      <c r="CC4" s="89"/>
-      <c r="CD4" s="89"/>
-      <c r="CE4" s="89"/>
-      <c r="CF4" s="89"/>
-      <c r="CG4" s="90"/>
-      <c r="CH4" s="88">
-        <f t="shared" ref="CH4" si="9">CL5</f>
+      <c r="CM5" s="12">
+        <f t="shared" ref="CM5" ca="1" si="29">CL5+1</f>
+        <v>45990</v>
+      </c>
+      <c r="CN5" s="12">
+        <f t="shared" ref="CN5" ca="1" si="30">CM5+1</f>
+        <v>45991</v>
+      </c>
+      <c r="CO5" s="12">
+        <f t="shared" ref="CO5" ca="1" si="31">CN5+1</f>
+        <v>45992</v>
+      </c>
+      <c r="CP5" s="12">
+        <f t="shared" ref="CP5" ca="1" si="32">CO5+1</f>
+        <v>45993</v>
+      </c>
+      <c r="CQ5" s="12">
+        <f t="shared" ref="CQ5" ca="1" si="33">CP5+1</f>
+        <v>45994</v>
+      </c>
+      <c r="CR5" s="12">
+        <f t="shared" ref="CR5" ca="1" si="34">CQ5+1</f>
+        <v>45995</v>
+      </c>
+      <c r="CS5" s="12">
+        <f t="shared" ref="CS5" ca="1" si="35">CR5+1</f>
         <v>45996</v>
       </c>
-      <c r="CI4" s="89"/>
-      <c r="CJ4" s="89"/>
-      <c r="CK4" s="89"/>
-      <c r="CL4" s="89"/>
-      <c r="CM4" s="89"/>
-      <c r="CN4" s="90"/>
-      <c r="CO4" s="88">
-        <f>CS5</f>
-        <v>46003</v>
-      </c>
-      <c r="CP4" s="89"/>
-      <c r="CQ4" s="89"/>
-      <c r="CR4" s="89"/>
-      <c r="CS4" s="89"/>
-      <c r="CT4" s="89"/>
-      <c r="CU4" s="90"/>
+      <c r="CT5" s="12">
+        <f t="shared" ref="CT5" ca="1" si="36">CS5+1</f>
+        <v>45997</v>
+      </c>
+      <c r="CU5" s="12">
+        <f t="shared" ref="CU5" ca="1" si="37">CT5+1</f>
+        <v>45998</v>
+      </c>
     </row>
-    <row r="5" spans="1:99" ht="15" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="59" t="s">
-        <v>7</v>
-      </c>
-      <c r="B5" s="94"/>
-      <c r="C5" s="94"/>
-      <c r="D5" s="94"/>
-      <c r="E5" s="94"/>
-      <c r="F5" s="94"/>
-      <c r="G5" s="94"/>
-      <c r="I5" s="11">
-        <f>Project_Start-WEEKDAY(Project_Start,1)+2+7*(Display_Week-1)</f>
-        <v>45915</v>
-      </c>
-      <c r="J5" s="10">
-        <f>I5+1</f>
-        <v>45916</v>
-      </c>
-      <c r="K5" s="10">
-        <f t="shared" ref="K5:AX5" si="10">J5+1</f>
-        <v>45917</v>
-      </c>
-      <c r="L5" s="10">
-        <f t="shared" si="10"/>
-        <v>45918</v>
-      </c>
-      <c r="M5" s="10">
-        <f t="shared" si="10"/>
-        <v>45919</v>
-      </c>
-      <c r="N5" s="10">
-        <f t="shared" si="10"/>
-        <v>45920</v>
-      </c>
-      <c r="O5" s="12">
-        <f t="shared" si="10"/>
-        <v>45921</v>
-      </c>
-      <c r="P5" s="11">
-        <f>O5+1</f>
-        <v>45922</v>
-      </c>
-      <c r="Q5" s="10">
-        <f>P5+1</f>
-        <v>45923</v>
-      </c>
-      <c r="R5" s="10">
-        <f t="shared" si="10"/>
-        <v>45924</v>
-      </c>
-      <c r="S5" s="10">
-        <f t="shared" si="10"/>
-        <v>45925</v>
-      </c>
-      <c r="T5" s="10">
-        <f t="shared" si="10"/>
-        <v>45926</v>
-      </c>
-      <c r="U5" s="10">
-        <f t="shared" si="10"/>
-        <v>45927</v>
-      </c>
-      <c r="V5" s="12">
-        <f t="shared" si="10"/>
-        <v>45928</v>
-      </c>
-      <c r="W5" s="11">
-        <f>V5+1</f>
-        <v>45929</v>
-      </c>
-      <c r="X5" s="10">
-        <f>W5+1</f>
-        <v>45930</v>
-      </c>
-      <c r="Y5" s="10">
-        <f t="shared" si="10"/>
-        <v>45931</v>
-      </c>
-      <c r="Z5" s="10">
-        <f t="shared" si="10"/>
-        <v>45932</v>
-      </c>
-      <c r="AA5" s="10">
-        <f t="shared" si="10"/>
-        <v>45933</v>
-      </c>
-      <c r="AB5" s="10">
-        <f t="shared" si="10"/>
-        <v>45934</v>
-      </c>
-      <c r="AC5" s="12">
-        <f t="shared" si="10"/>
-        <v>45935</v>
-      </c>
-      <c r="AD5" s="11">
-        <f>AC5+1</f>
-        <v>45936</v>
-      </c>
-      <c r="AE5" s="10">
-        <f>AD5+1</f>
-        <v>45937</v>
-      </c>
-      <c r="AF5" s="10">
-        <f t="shared" si="10"/>
-        <v>45938</v>
-      </c>
-      <c r="AG5" s="10">
-        <f t="shared" si="10"/>
-        <v>45939</v>
-      </c>
-      <c r="AH5" s="10">
-        <f t="shared" si="10"/>
-        <v>45940</v>
-      </c>
-      <c r="AI5" s="10">
-        <f t="shared" si="10"/>
-        <v>45941</v>
-      </c>
-      <c r="AJ5" s="12">
-        <f t="shared" si="10"/>
-        <v>45942</v>
-      </c>
-      <c r="AK5" s="11">
-        <f>AJ5+1</f>
-        <v>45943</v>
-      </c>
-      <c r="AL5" s="10">
-        <f>AK5+1</f>
-        <v>45944</v>
-      </c>
-      <c r="AM5" s="10">
-        <f t="shared" si="10"/>
-        <v>45945</v>
-      </c>
-      <c r="AN5" s="10">
-        <f t="shared" si="10"/>
-        <v>45946</v>
-      </c>
-      <c r="AO5" s="10">
-        <f t="shared" si="10"/>
-        <v>45947</v>
-      </c>
-      <c r="AP5" s="10">
-        <f t="shared" si="10"/>
-        <v>45948</v>
-      </c>
-      <c r="AQ5" s="12">
-        <f t="shared" si="10"/>
-        <v>45949</v>
-      </c>
-      <c r="AR5" s="11">
-        <f>AQ5+1</f>
-        <v>45950</v>
-      </c>
-      <c r="AS5" s="10">
-        <f>AR5+1</f>
-        <v>45951</v>
-      </c>
-      <c r="AT5" s="10">
-        <f t="shared" si="10"/>
-        <v>45952</v>
-      </c>
-      <c r="AU5" s="10">
-        <f t="shared" si="10"/>
-        <v>45953</v>
-      </c>
-      <c r="AV5" s="10">
-        <f t="shared" si="10"/>
-        <v>45954</v>
-      </c>
-      <c r="AW5" s="10">
-        <f t="shared" si="10"/>
-        <v>45955</v>
-      </c>
-      <c r="AX5" s="12">
-        <f t="shared" si="10"/>
-        <v>45956</v>
-      </c>
-      <c r="AY5" s="11">
-        <f>AX5+1</f>
-        <v>45957</v>
-      </c>
-      <c r="AZ5" s="10">
-        <f>AY5+1</f>
-        <v>45958</v>
-      </c>
-      <c r="BA5" s="10">
-        <f t="shared" ref="BA5:BE5" si="11">AZ5+1</f>
-        <v>45959</v>
-      </c>
-      <c r="BB5" s="10">
-        <f t="shared" si="11"/>
-        <v>45960</v>
-      </c>
-      <c r="BC5" s="10">
-        <f t="shared" si="11"/>
-        <v>45961</v>
-      </c>
-      <c r="BD5" s="10">
-        <f t="shared" si="11"/>
-        <v>45962</v>
-      </c>
-      <c r="BE5" s="12">
-        <f t="shared" si="11"/>
-        <v>45963</v>
-      </c>
-      <c r="BF5" s="11">
-        <f>BE5+1</f>
-        <v>45964</v>
-      </c>
-      <c r="BG5" s="10">
-        <f>BF5+1</f>
-        <v>45965</v>
-      </c>
-      <c r="BH5" s="10">
-        <f t="shared" ref="BH5:BL5" si="12">BG5+1</f>
-        <v>45966</v>
-      </c>
-      <c r="BI5" s="10">
-        <f t="shared" si="12"/>
-        <v>45967</v>
-      </c>
-      <c r="BJ5" s="10">
-        <f t="shared" si="12"/>
-        <v>45968</v>
-      </c>
-      <c r="BK5" s="10">
-        <f t="shared" si="12"/>
-        <v>45969</v>
-      </c>
-      <c r="BL5" s="12">
-        <f t="shared" si="12"/>
-        <v>45970</v>
-      </c>
-      <c r="BM5" s="12">
-        <f t="shared" ref="BM5" si="13">BL5+1</f>
-        <v>45971</v>
-      </c>
-      <c r="BN5" s="12">
-        <f t="shared" ref="BN5" si="14">BM5+1</f>
-        <v>45972</v>
-      </c>
-      <c r="BO5" s="12">
-        <f t="shared" ref="BO5" si="15">BN5+1</f>
-        <v>45973</v>
-      </c>
-      <c r="BP5" s="12">
-        <f t="shared" ref="BP5" si="16">BO5+1</f>
-        <v>45974</v>
-      </c>
-      <c r="BQ5" s="12">
-        <f t="shared" ref="BQ5" si="17">BP5+1</f>
-        <v>45975</v>
-      </c>
-      <c r="BR5" s="12">
-        <f t="shared" ref="BR5" si="18">BQ5+1</f>
-        <v>45976</v>
-      </c>
-      <c r="BS5" s="12">
-        <f t="shared" ref="BS5" si="19">BR5+1</f>
-        <v>45977</v>
-      </c>
-      <c r="BT5" s="12">
-        <f t="shared" ref="BT5" si="20">BS5+1</f>
-        <v>45978</v>
-      </c>
-      <c r="BU5" s="12">
-        <f t="shared" ref="BU5" si="21">BT5+1</f>
-        <v>45979</v>
-      </c>
-      <c r="BV5" s="12">
-        <f t="shared" ref="BV5" si="22">BU5+1</f>
-        <v>45980</v>
-      </c>
-      <c r="BW5" s="12">
-        <f t="shared" ref="BW5" si="23">BV5+1</f>
-        <v>45981</v>
-      </c>
-      <c r="BX5" s="12">
-        <f t="shared" ref="BX5" si="24">BW5+1</f>
-        <v>45982</v>
-      </c>
-      <c r="BY5" s="12">
-        <f t="shared" ref="BY5" si="25">BX5+1</f>
-        <v>45983</v>
-      </c>
-      <c r="BZ5" s="12">
-        <f t="shared" ref="BZ5" si="26">BY5+1</f>
-        <v>45984</v>
-      </c>
-      <c r="CA5" s="12">
-        <f t="shared" ref="CA5" si="27">BZ5+1</f>
-        <v>45985</v>
-      </c>
-      <c r="CB5" s="12">
-        <f t="shared" ref="CB5" si="28">CA5+1</f>
-        <v>45986</v>
-      </c>
-      <c r="CC5" s="12">
-        <f t="shared" ref="CC5" si="29">CB5+1</f>
-        <v>45987</v>
-      </c>
-      <c r="CD5" s="12">
-        <f t="shared" ref="CD5" si="30">CC5+1</f>
-        <v>45988</v>
-      </c>
-      <c r="CE5" s="12">
-        <f t="shared" ref="CE5" si="31">CD5+1</f>
-        <v>45989</v>
-      </c>
-      <c r="CF5" s="12">
-        <f t="shared" ref="CF5" si="32">CE5+1</f>
-        <v>45990</v>
-      </c>
-      <c r="CG5" s="12">
-        <f t="shared" ref="CG5" si="33">CF5+1</f>
-        <v>45991</v>
-      </c>
-      <c r="CH5" s="12">
-        <f t="shared" ref="CH5" si="34">CG5+1</f>
-        <v>45992</v>
-      </c>
-      <c r="CI5" s="12">
-        <f t="shared" ref="CI5" si="35">CH5+1</f>
-        <v>45993</v>
-      </c>
-      <c r="CJ5" s="12">
-        <f t="shared" ref="CJ5" si="36">CI5+1</f>
-        <v>45994</v>
-      </c>
-      <c r="CK5" s="12">
-        <f t="shared" ref="CK5" si="37">CJ5+1</f>
-        <v>45995</v>
-      </c>
-      <c r="CL5" s="12">
-        <f t="shared" ref="CL5" si="38">CK5+1</f>
-        <v>45996</v>
-      </c>
-      <c r="CM5" s="12">
-        <f t="shared" ref="CM5" si="39">CL5+1</f>
-        <v>45997</v>
-      </c>
-      <c r="CN5" s="12">
-        <f t="shared" ref="CN5" si="40">CM5+1</f>
-        <v>45998</v>
-      </c>
-      <c r="CO5" s="12">
-        <f t="shared" ref="CO5" si="41">CN5+1</f>
-        <v>45999</v>
-      </c>
-      <c r="CP5" s="12">
-        <f t="shared" ref="CP5" si="42">CO5+1</f>
-        <v>46000</v>
-      </c>
-      <c r="CQ5" s="12">
-        <f t="shared" ref="CQ5" si="43">CP5+1</f>
-        <v>46001</v>
-      </c>
-      <c r="CR5" s="12">
-        <f t="shared" ref="CR5" si="44">CQ5+1</f>
-        <v>46002</v>
-      </c>
-      <c r="CS5" s="12">
-        <f t="shared" ref="CS5" si="45">CR5+1</f>
-        <v>46003</v>
-      </c>
-      <c r="CT5" s="12">
-        <f t="shared" ref="CT5" si="46">CS5+1</f>
-        <v>46004</v>
-      </c>
-      <c r="CU5" s="12">
-        <f t="shared" ref="CU5" si="47">CT5+1</f>
-        <v>46005</v>
-      </c>
-    </row>
-    <row r="6" spans="1:99" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:99" ht="30" customHeight="1" thickBot="1">
       <c r="A6" s="59" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G6" s="9"/>
       <c r="H6" s="9" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I6" s="13" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J6" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="K6" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="L6" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="M6" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="N6" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="O6" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="P6" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="K6" s="13" t="s">
+      <c r="Q6" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="L6" s="13" t="s">
+      <c r="R6" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="S6" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="T6" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="U6" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="V6" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="W6" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="M6" s="13" t="s">
+      <c r="X6" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="Y6" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="N6" s="13" t="s">
+      <c r="Z6" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="AA6" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="O6" s="13" t="s">
+      <c r="AB6" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="AC6" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="AD6" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="AE6" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="AF6" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="AG6" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="AH6" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="P6" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q6" s="13" t="s">
+      <c r="AI6" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="AJ6" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="AK6" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="R6" s="13" t="s">
+      <c r="AL6" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="S6" s="13" t="s">
+      <c r="AM6" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="AN6" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="AO6" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="AP6" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="AQ6" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="AR6" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="T6" s="13" t="s">
+      <c r="AS6" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="AT6" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="U6" s="13" t="s">
+      <c r="AU6" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="AV6" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="V6" s="13" t="s">
+      <c r="AW6" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="AX6" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="AY6" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="AZ6" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="BA6" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="BB6" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="BC6" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="W6" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="X6" s="13" t="s">
+      <c r="BD6" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="BE6" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="BF6" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="Y6" s="13" t="s">
+      <c r="BG6" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="Z6" s="13" t="s">
+      <c r="BH6" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="BI6" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="BJ6" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="BK6" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="BL6" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="BM6" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="AA6" s="13" t="s">
+      <c r="BN6" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="BO6" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="AB6" s="13" t="s">
+      <c r="BP6" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="BQ6" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="AC6" s="13" t="s">
+      <c r="BR6" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="BS6" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="BT6" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="BU6" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="BV6" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="BW6" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="BX6" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="AD6" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="AE6" s="13" t="s">
+      <c r="BY6" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="BZ6" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="CA6" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="AF6" s="13" t="s">
+      <c r="CB6" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="AG6" s="13" t="s">
+      <c r="CC6" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="CD6" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="CE6" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="CF6" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="CG6" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="CH6" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="AH6" s="13" t="s">
+      <c r="CI6" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="CJ6" s="13" t="s">
         <v>18</v>
       </c>
-      <c r="AI6" s="13" t="s">
+      <c r="CK6" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="CL6" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="AJ6" s="13" t="s">
+      <c r="CM6" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="CN6" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="CO6" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="CP6" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="CQ6" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="CR6" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="CS6" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="AK6" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="AL6" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="AM6" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="AN6" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="AO6" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="AP6" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="AQ6" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="AR6" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="AS6" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="AT6" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="AU6" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="AV6" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="AW6" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="AX6" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="AY6" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="AZ6" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="BA6" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="BB6" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="BC6" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="BD6" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="BE6" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="BF6" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="BG6" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="BH6" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="BI6" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="BJ6" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="BK6" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="BL6" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="BM6" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="BN6" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="BO6" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="BP6" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="BQ6" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="BR6" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="BS6" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="BT6" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="BU6" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="BV6" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="BW6" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="BX6" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="BY6" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="BZ6" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="CA6" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="CB6" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="CC6" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="CD6" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="CE6" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="CF6" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="CG6" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="CH6" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="CI6" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="CJ6" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="CK6" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="CL6" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="CM6" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="CN6" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="CO6" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="CP6" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="CQ6" s="13" t="s">
-        <v>17</v>
-      </c>
-      <c r="CR6" s="13" t="s">
-        <v>16</v>
-      </c>
-      <c r="CS6" s="13" t="s">
-        <v>18</v>
-      </c>
       <c r="CT6" s="13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="CU6" s="13" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:99" ht="30" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:99" ht="30" hidden="1" customHeight="1" thickBot="1">
       <c r="A7" s="58" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C7" s="62"/>
       <c r="E7"/>
       <c r="H7" t="str">
-        <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+        <f ca="1">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v/>
       </c>
       <c r="I7" s="44"/>
@@ -2477,12 +2438,12 @@
       <c r="BK7" s="44"/>
       <c r="BL7" s="44"/>
     </row>
-    <row r="8" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A8" s="59" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>52</v>
+        <v>23</v>
       </c>
       <c r="C8" s="69"/>
       <c r="D8" s="19"/>
@@ -2490,7 +2451,7 @@
       <c r="F8" s="21"/>
       <c r="G8" s="17"/>
       <c r="H8" s="17" t="str">
-        <f t="shared" ref="H8:H36" si="48">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+        <f t="shared" ref="H8:H33" ca="1" si="38">IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
         <v/>
       </c>
       <c r="I8" s="44"/>
@@ -2585,31 +2546,31 @@
       <c r="CT8" s="44"/>
       <c r="CU8" s="44"/>
     </row>
-    <row r="9" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A9" s="59" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B9" s="78" t="s">
-        <v>56</v>
+        <v>25</v>
       </c>
       <c r="C9" s="70" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
       <c r="D9" s="22">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="E9" s="83">
-        <f>Project_Start</f>
-        <v>45919</v>
+        <f ca="1">Project_Start</f>
+        <v>45909</v>
       </c>
       <c r="F9" s="83">
-        <f>E9+9</f>
-        <v>45928</v>
+        <f ca="1">E9+3</f>
+        <v>45912</v>
       </c>
       <c r="G9" s="17"/>
       <c r="H9" s="17">
-        <f t="shared" si="48"/>
-        <v>10</v>
+        <f t="shared" ca="1" si="38"/>
+        <v>4</v>
       </c>
       <c r="I9" s="44"/>
       <c r="J9" s="44"/>
@@ -2703,31 +2664,29 @@
       <c r="CT9" s="44"/>
       <c r="CU9" s="44"/>
     </row>
-    <row r="10" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A10" s="59" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="B10" s="78" t="s">
-        <v>53</v>
-      </c>
-      <c r="C10" s="70" t="s">
-        <v>61</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="C10" s="70"/>
       <c r="D10" s="22">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="E10" s="83">
-        <f>F9+1</f>
-        <v>45929</v>
+        <f ca="1">Project_Start</f>
+        <v>45909</v>
       </c>
       <c r="F10" s="83">
-        <f>E10+6</f>
-        <v>45935</v>
+        <f t="shared" ref="F10:F13" ca="1" si="39">E10+3</f>
+        <v>45912</v>
       </c>
       <c r="G10" s="17"/>
       <c r="H10" s="17">
-        <f t="shared" si="48"/>
-        <v>7</v>
+        <f t="shared" ca="1" si="38"/>
+        <v>4</v>
       </c>
       <c r="I10" s="44"/>
       <c r="J10" s="44"/>
@@ -2821,29 +2780,27 @@
       <c r="CT10" s="44"/>
       <c r="CU10" s="44"/>
     </row>
-    <row r="11" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A11" s="58"/>
       <c r="B11" s="78" t="s">
-        <v>54</v>
-      </c>
-      <c r="C11" s="70" t="s">
-        <v>61</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="C11" s="70"/>
       <c r="D11" s="22">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="E11" s="83">
-        <f>Project_Start+7</f>
-        <v>45926</v>
+        <f ca="1">Project_Start</f>
+        <v>45909</v>
       </c>
       <c r="F11" s="83">
-        <f>E11+5</f>
-        <v>45931</v>
+        <f t="shared" ca="1" si="39"/>
+        <v>45912</v>
       </c>
       <c r="G11" s="17"/>
       <c r="H11" s="17">
-        <f t="shared" si="48"/>
-        <v>6</v>
+        <f t="shared" ca="1" si="38"/>
+        <v>4</v>
       </c>
       <c r="I11" s="44"/>
       <c r="J11" s="44"/>
@@ -2937,29 +2894,27 @@
       <c r="CT11" s="44"/>
       <c r="CU11" s="44"/>
     </row>
-    <row r="12" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A12" s="58"/>
       <c r="B12" s="78" t="s">
-        <v>55</v>
-      </c>
-      <c r="C12" s="70" t="s">
-        <v>62</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="C12" s="70"/>
       <c r="D12" s="22">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="E12" s="83">
-        <f>F10+5</f>
-        <v>45940</v>
+        <f ca="1">Project_Start</f>
+        <v>45909</v>
       </c>
       <c r="F12" s="83">
-        <f>E12+7</f>
-        <v>45947</v>
+        <f t="shared" ca="1" si="39"/>
+        <v>45912</v>
       </c>
       <c r="G12" s="17"/>
       <c r="H12" s="17">
-        <f t="shared" si="48"/>
-        <v>8</v>
+        <f t="shared" ca="1" si="38"/>
+        <v>4</v>
       </c>
       <c r="I12" s="44"/>
       <c r="J12" s="44"/>
@@ -3053,29 +3008,25 @@
       <c r="CT12" s="44"/>
       <c r="CU12" s="44"/>
     </row>
-    <row r="13" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A13" s="58"/>
       <c r="B13" s="78" t="s">
-        <v>59</v>
-      </c>
-      <c r="C13" s="70" t="s">
-        <v>60</v>
-      </c>
-      <c r="D13" s="22">
-        <v>0</v>
-      </c>
+        <v>31</v>
+      </c>
+      <c r="C13" s="70"/>
+      <c r="D13" s="22"/>
       <c r="E13" s="83">
-        <f>F12</f>
-        <v>45947</v>
+        <f ca="1">Project_Start</f>
+        <v>45909</v>
       </c>
       <c r="F13" s="83">
-        <f>E13+7</f>
-        <v>45954</v>
+        <f t="shared" ca="1" si="39"/>
+        <v>45912</v>
       </c>
       <c r="G13" s="17"/>
       <c r="H13" s="17">
-        <f t="shared" si="48"/>
-        <v>8</v>
+        <f t="shared" ca="1" si="38"/>
+        <v>4</v>
       </c>
       <c r="I13" s="44"/>
       <c r="J13" s="44"/>
@@ -3169,27 +3120,21 @@
       <c r="CT13" s="44"/>
       <c r="CU13" s="44"/>
     </row>
-    <row r="14" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A14" s="58"/>
-      <c r="B14" s="86" t="s">
-        <v>58</v>
-      </c>
-      <c r="C14" s="70" t="s">
-        <v>60</v>
-      </c>
-      <c r="D14" s="22">
-        <v>0</v>
-      </c>
-      <c r="E14" s="85">
-        <v>45961</v>
-      </c>
-      <c r="F14" s="85">
-        <v>45961</v>
-      </c>
+    <row r="14" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1">
+      <c r="A14" s="59" t="s">
+        <v>32</v>
+      </c>
+      <c r="B14" s="23" t="s">
+        <v>33</v>
+      </c>
+      <c r="C14" s="71"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="25"/>
+      <c r="F14" s="26"/>
       <c r="G14" s="17"/>
-      <c r="H14" s="17">
-        <f t="shared" si="48"/>
-        <v>1</v>
+      <c r="H14" s="17" t="str">
+        <f t="shared" ca="1" si="38"/>
+        <v/>
       </c>
       <c r="I14" s="44"/>
       <c r="J14" s="44"/>
@@ -3283,28 +3228,27 @@
       <c r="CT14" s="44"/>
       <c r="CU14" s="44"/>
     </row>
-    <row r="15" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A15" s="58"/>
-      <c r="B15" s="78" t="s">
-        <v>57</v>
-      </c>
-      <c r="C15" s="70" t="s">
-        <v>60</v>
-      </c>
-      <c r="D15" s="22">
-        <v>0</v>
-      </c>
-      <c r="E15" s="83">
-        <v>45947</v>
-      </c>
-      <c r="F15" s="83">
-        <f>E15+23</f>
-        <v>45970</v>
+    <row r="15" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1">
+      <c r="A15" s="59"/>
+      <c r="B15" s="79" t="s">
+        <v>34</v>
+      </c>
+      <c r="C15" s="72"/>
+      <c r="D15" s="27">
+        <v>0.5</v>
+      </c>
+      <c r="E15" s="84">
+        <f ca="1">E13+1</f>
+        <v>45910</v>
+      </c>
+      <c r="F15" s="84">
+        <f ca="1">E15+4</f>
+        <v>45914</v>
       </c>
       <c r="G15" s="17"/>
       <c r="H15" s="17">
-        <f t="shared" si="48"/>
-        <v>24</v>
+        <f t="shared" ca="1" si="38"/>
+        <v>5</v>
       </c>
       <c r="I15" s="44"/>
       <c r="J15" s="44"/>
@@ -3398,28 +3342,27 @@
       <c r="CT15" s="44"/>
       <c r="CU15" s="44"/>
     </row>
-    <row r="16" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A16" s="58"/>
-      <c r="B16" s="86" t="s">
-        <v>63</v>
-      </c>
-      <c r="C16" s="70" t="s">
-        <v>60</v>
-      </c>
-      <c r="D16" s="22">
-        <v>0</v>
-      </c>
-      <c r="E16" s="87">
-        <f>F16</f>
-        <v>45975</v>
-      </c>
-      <c r="F16" s="85">
-        <v>45975</v>
+      <c r="B16" s="79" t="s">
+        <v>35</v>
+      </c>
+      <c r="C16" s="72"/>
+      <c r="D16" s="27">
+        <v>0.5</v>
+      </c>
+      <c r="E16" s="84">
+        <f t="shared" ref="E16:E19" si="40">E14+1</f>
+        <v>1</v>
+      </c>
+      <c r="F16" s="84">
+        <f t="shared" ref="F16:F19" si="41">E16+4</f>
+        <v>5</v>
       </c>
       <c r="G16" s="17"/>
       <c r="H16" s="17">
-        <f t="shared" si="48"/>
-        <v>1</v>
+        <f t="shared" ca="1" si="38"/>
+        <v>5</v>
       </c>
       <c r="I16" s="44"/>
       <c r="J16" s="44"/>
@@ -3433,8 +3376,8 @@
       <c r="R16" s="44"/>
       <c r="S16" s="44"/>
       <c r="T16" s="44"/>
-      <c r="U16" s="44"/>
-      <c r="V16" s="44"/>
+      <c r="U16" s="45"/>
+      <c r="V16" s="45"/>
       <c r="W16" s="44"/>
       <c r="X16" s="44"/>
       <c r="Y16" s="44"/>
@@ -3513,21 +3456,25 @@
       <c r="CT16" s="44"/>
       <c r="CU16" s="44"/>
     </row>
-    <row r="17" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A17" s="59" t="s">
-        <v>27</v>
-      </c>
-      <c r="B17" s="23" t="s">
-        <v>64</v>
-      </c>
-      <c r="C17" s="71"/>
-      <c r="D17" s="24"/>
-      <c r="E17" s="25"/>
-      <c r="F17" s="26"/>
+    <row r="17" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1">
+      <c r="A17" s="58"/>
+      <c r="B17" s="79" t="s">
+        <v>29</v>
+      </c>
+      <c r="C17" s="72"/>
+      <c r="D17" s="27"/>
+      <c r="E17" s="84">
+        <f t="shared" ca="1" si="40"/>
+        <v>45911</v>
+      </c>
+      <c r="F17" s="84">
+        <f t="shared" ca="1" si="41"/>
+        <v>45915</v>
+      </c>
       <c r="G17" s="17"/>
-      <c r="H17" s="17" t="str">
-        <f t="shared" si="48"/>
-        <v/>
+      <c r="H17" s="17">
+        <f t="shared" ca="1" si="38"/>
+        <v>5</v>
       </c>
       <c r="I17" s="44"/>
       <c r="J17" s="44"/>
@@ -3621,26 +3568,24 @@
       <c r="CT17" s="44"/>
       <c r="CU17" s="44"/>
     </row>
-    <row r="18" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A18" s="59"/>
+    <row r="18" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1">
+      <c r="A18" s="58"/>
       <c r="B18" s="79" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C18" s="72"/>
-      <c r="D18" s="27">
-        <v>0</v>
-      </c>
+      <c r="D18" s="27"/>
       <c r="E18" s="84">
-        <f>E16+1</f>
-        <v>45976</v>
+        <f t="shared" si="40"/>
+        <v>2</v>
       </c>
       <c r="F18" s="84">
-        <f>E18+4</f>
-        <v>45980</v>
+        <f t="shared" si="41"/>
+        <v>6</v>
       </c>
       <c r="G18" s="17"/>
       <c r="H18" s="17">
-        <f t="shared" si="48"/>
+        <f t="shared" ca="1" si="38"/>
         <v>5</v>
       </c>
       <c r="I18" s="44"/>
@@ -3659,7 +3604,7 @@
       <c r="V18" s="44"/>
       <c r="W18" s="44"/>
       <c r="X18" s="44"/>
-      <c r="Y18" s="44"/>
+      <c r="Y18" s="45"/>
       <c r="Z18" s="44"/>
       <c r="AA18" s="44"/>
       <c r="AB18" s="44"/>
@@ -3735,26 +3680,24 @@
       <c r="CT18" s="44"/>
       <c r="CU18" s="44"/>
     </row>
-    <row r="19" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A19" s="58"/>
       <c r="B19" s="79" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C19" s="72"/>
-      <c r="D19" s="27">
-        <v>0</v>
-      </c>
+      <c r="D19" s="27"/>
       <c r="E19" s="84">
-        <f t="shared" ref="E19:E22" si="49">E17+1</f>
-        <v>1</v>
+        <f t="shared" ca="1" si="40"/>
+        <v>45912</v>
       </c>
       <c r="F19" s="84">
-        <f t="shared" ref="F19:F22" si="50">E19+4</f>
-        <v>5</v>
+        <f t="shared" ca="1" si="41"/>
+        <v>45916</v>
       </c>
       <c r="G19" s="17"/>
       <c r="H19" s="17">
-        <f t="shared" si="48"/>
+        <f t="shared" ca="1" si="38"/>
         <v>5</v>
       </c>
       <c r="I19" s="44"/>
@@ -3769,8 +3712,8 @@
       <c r="R19" s="44"/>
       <c r="S19" s="44"/>
       <c r="T19" s="44"/>
-      <c r="U19" s="45"/>
-      <c r="V19" s="45"/>
+      <c r="U19" s="44"/>
+      <c r="V19" s="44"/>
       <c r="W19" s="44"/>
       <c r="X19" s="44"/>
       <c r="Y19" s="44"/>
@@ -3849,27 +3792,21 @@
       <c r="CT19" s="44"/>
       <c r="CU19" s="44"/>
     </row>
-    <row r="20" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A20" s="58"/>
-      <c r="B20" s="79" t="s">
-        <v>24</v>
-      </c>
-      <c r="C20" s="72"/>
-      <c r="D20" s="27">
-        <v>0</v>
-      </c>
-      <c r="E20" s="84">
-        <f t="shared" si="49"/>
-        <v>45977</v>
-      </c>
-      <c r="F20" s="84">
-        <f t="shared" si="50"/>
-        <v>45981</v>
-      </c>
+    <row r="20" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1">
+      <c r="A20" s="58" t="s">
+        <v>36</v>
+      </c>
+      <c r="B20" s="28" t="s">
+        <v>37</v>
+      </c>
+      <c r="C20" s="73"/>
+      <c r="D20" s="29"/>
+      <c r="E20" s="30"/>
+      <c r="F20" s="31"/>
       <c r="G20" s="17"/>
-      <c r="H20" s="17">
-        <f t="shared" si="48"/>
-        <v>5</v>
+      <c r="H20" s="17" t="str">
+        <f t="shared" ca="1" si="38"/>
+        <v/>
       </c>
       <c r="I20" s="44"/>
       <c r="J20" s="44"/>
@@ -3963,27 +3900,25 @@
       <c r="CT20" s="44"/>
       <c r="CU20" s="44"/>
     </row>
-    <row r="21" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A21" s="58"/>
-      <c r="B21" s="79" t="s">
-        <v>25</v>
-      </c>
-      <c r="C21" s="72"/>
-      <c r="D21" s="27">
-        <v>0</v>
-      </c>
-      <c r="E21" s="84">
-        <f t="shared" si="49"/>
-        <v>2</v>
-      </c>
-      <c r="F21" s="84">
-        <f t="shared" si="50"/>
-        <v>6</v>
+      <c r="B21" s="80" t="s">
+        <v>34</v>
+      </c>
+      <c r="C21" s="74"/>
+      <c r="D21" s="32"/>
+      <c r="E21" s="66">
+        <f ca="1">E9+15</f>
+        <v>45924</v>
+      </c>
+      <c r="F21" s="66">
+        <f ca="1">E21+5</f>
+        <v>45929</v>
       </c>
       <c r="G21" s="17"/>
       <c r="H21" s="17">
-        <f t="shared" si="48"/>
-        <v>5</v>
+        <f t="shared" ca="1" si="38"/>
+        <v>6</v>
       </c>
       <c r="I21" s="44"/>
       <c r="J21" s="44"/>
@@ -4001,7 +3936,7 @@
       <c r="V21" s="44"/>
       <c r="W21" s="44"/>
       <c r="X21" s="44"/>
-      <c r="Y21" s="45"/>
+      <c r="Y21" s="44"/>
       <c r="Z21" s="44"/>
       <c r="AA21" s="44"/>
       <c r="AB21" s="44"/>
@@ -4077,26 +4012,24 @@
       <c r="CT21" s="44"/>
       <c r="CU21" s="44"/>
     </row>
-    <row r="22" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A22" s="58"/>
-      <c r="B22" s="79" t="s">
-        <v>26</v>
-      </c>
-      <c r="C22" s="72"/>
-      <c r="D22" s="27">
-        <v>0</v>
-      </c>
-      <c r="E22" s="84">
-        <f t="shared" si="49"/>
-        <v>45978</v>
-      </c>
-      <c r="F22" s="84">
-        <f t="shared" si="50"/>
-        <v>45982</v>
+      <c r="B22" s="80" t="s">
+        <v>35</v>
+      </c>
+      <c r="C22" s="74"/>
+      <c r="D22" s="32"/>
+      <c r="E22" s="66">
+        <f ca="1">F21+1</f>
+        <v>45930</v>
+      </c>
+      <c r="F22" s="66">
+        <f ca="1">E22+4</f>
+        <v>45934</v>
       </c>
       <c r="G22" s="17"/>
       <c r="H22" s="17">
-        <f t="shared" si="48"/>
+        <f t="shared" ca="1" si="38"/>
         <v>5</v>
       </c>
       <c r="I22" s="44"/>
@@ -4191,21 +4124,25 @@
       <c r="CT22" s="44"/>
       <c r="CU22" s="44"/>
     </row>
-    <row r="23" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A23" s="58" t="s">
-        <v>30</v>
-      </c>
-      <c r="B23" s="28" t="s">
-        <v>31</v>
-      </c>
-      <c r="C23" s="73"/>
-      <c r="D23" s="29"/>
-      <c r="E23" s="30"/>
-      <c r="F23" s="31"/>
+    <row r="23" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1">
+      <c r="A23" s="58"/>
+      <c r="B23" s="80" t="s">
+        <v>29</v>
+      </c>
+      <c r="C23" s="74"/>
+      <c r="D23" s="32"/>
+      <c r="E23" s="66">
+        <f ca="1">E22+5</f>
+        <v>45935</v>
+      </c>
+      <c r="F23" s="66">
+        <f ca="1">E23+5</f>
+        <v>45940</v>
+      </c>
       <c r="G23" s="17"/>
-      <c r="H23" s="17" t="str">
-        <f t="shared" si="48"/>
-        <v/>
+      <c r="H23" s="17">
+        <f t="shared" ca="1" si="38"/>
+        <v>6</v>
       </c>
       <c r="I23" s="44"/>
       <c r="J23" s="44"/>
@@ -4299,25 +4236,25 @@
       <c r="CT23" s="44"/>
       <c r="CU23" s="44"/>
     </row>
-    <row r="24" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A24" s="58"/>
       <c r="B24" s="80" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C24" s="74"/>
       <c r="D24" s="32"/>
       <c r="E24" s="66">
-        <f>E9+15</f>
-        <v>45934</v>
+        <f ca="1">F23+1</f>
+        <v>45941</v>
       </c>
       <c r="F24" s="66">
-        <f>E24+5</f>
-        <v>45939</v>
+        <f ca="1">E24+4</f>
+        <v>45945</v>
       </c>
       <c r="G24" s="17"/>
       <c r="H24" s="17">
-        <f t="shared" si="48"/>
-        <v>6</v>
+        <f t="shared" ca="1" si="38"/>
+        <v>5</v>
       </c>
       <c r="I24" s="44"/>
       <c r="J24" s="44"/>
@@ -4411,24 +4348,24 @@
       <c r="CT24" s="44"/>
       <c r="CU24" s="44"/>
     </row>
-    <row r="25" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A25" s="58"/>
       <c r="B25" s="80" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C25" s="74"/>
       <c r="D25" s="32"/>
       <c r="E25" s="66">
-        <f>F24+1</f>
-        <v>45940</v>
+        <f ca="1">E23</f>
+        <v>45935</v>
       </c>
       <c r="F25" s="66">
-        <f>E25+4</f>
-        <v>45944</v>
+        <f ca="1">E25+4</f>
+        <v>45939</v>
       </c>
       <c r="G25" s="17"/>
       <c r="H25" s="17">
-        <f t="shared" si="48"/>
+        <f t="shared" ca="1" si="38"/>
         <v>5</v>
       </c>
       <c r="I25" s="44"/>
@@ -4523,25 +4460,21 @@
       <c r="CT25" s="44"/>
       <c r="CU25" s="44"/>
     </row>
-    <row r="26" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A26" s="58"/>
-      <c r="B26" s="80" t="s">
-        <v>24</v>
-      </c>
-      <c r="C26" s="74"/>
-      <c r="D26" s="32"/>
-      <c r="E26" s="66">
-        <f>E25+5</f>
-        <v>45945</v>
-      </c>
-      <c r="F26" s="66">
-        <f>E26+5</f>
-        <v>45950</v>
-      </c>
+    <row r="26" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1">
+      <c r="A26" s="58" t="s">
+        <v>36</v>
+      </c>
+      <c r="B26" s="33" t="s">
+        <v>38</v>
+      </c>
+      <c r="C26" s="75"/>
+      <c r="D26" s="34"/>
+      <c r="E26" s="35"/>
+      <c r="F26" s="36"/>
       <c r="G26" s="17"/>
-      <c r="H26" s="17">
-        <f t="shared" si="48"/>
-        <v>6</v>
+      <c r="H26" s="17" t="str">
+        <f t="shared" ca="1" si="38"/>
+        <v/>
       </c>
       <c r="I26" s="44"/>
       <c r="J26" s="44"/>
@@ -4635,25 +4568,23 @@
       <c r="CT26" s="44"/>
       <c r="CU26" s="44"/>
     </row>
-    <row r="27" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A27" s="58"/>
-      <c r="B27" s="80" t="s">
-        <v>25</v>
-      </c>
-      <c r="C27" s="74"/>
-      <c r="D27" s="32"/>
-      <c r="E27" s="66">
-        <f>F26+1</f>
-        <v>45951</v>
-      </c>
-      <c r="F27" s="66">
-        <f>E27+4</f>
-        <v>45955</v>
+      <c r="B27" s="81" t="s">
+        <v>34</v>
+      </c>
+      <c r="C27" s="76"/>
+      <c r="D27" s="37"/>
+      <c r="E27" s="67" t="s">
+        <v>39</v>
+      </c>
+      <c r="F27" s="67" t="s">
+        <v>39</v>
       </c>
       <c r="G27" s="17"/>
-      <c r="H27" s="17">
-        <f t="shared" si="48"/>
-        <v>5</v>
+      <c r="H27" s="17" t="e">
+        <f t="shared" ca="1" si="38"/>
+        <v>#VALUE!</v>
       </c>
       <c r="I27" s="44"/>
       <c r="J27" s="44"/>
@@ -4747,25 +4678,23 @@
       <c r="CT27" s="44"/>
       <c r="CU27" s="44"/>
     </row>
-    <row r="28" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A28" s="58"/>
-      <c r="B28" s="80" t="s">
-        <v>26</v>
-      </c>
-      <c r="C28" s="74"/>
-      <c r="D28" s="32"/>
-      <c r="E28" s="66">
-        <f>E26</f>
-        <v>45945</v>
-      </c>
-      <c r="F28" s="66">
-        <f>E28+4</f>
-        <v>45949</v>
+      <c r="B28" s="81" t="s">
+        <v>35</v>
+      </c>
+      <c r="C28" s="76"/>
+      <c r="D28" s="37"/>
+      <c r="E28" s="67" t="s">
+        <v>39</v>
+      </c>
+      <c r="F28" s="67" t="s">
+        <v>39</v>
       </c>
       <c r="G28" s="17"/>
-      <c r="H28" s="17">
-        <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
-        <v>5</v>
+      <c r="H28" s="17" t="e">
+        <f t="shared" ca="1" si="38"/>
+        <v>#VALUE!</v>
       </c>
       <c r="I28" s="44"/>
       <c r="J28" s="44"/>
@@ -4859,21 +4788,23 @@
       <c r="CT28" s="44"/>
       <c r="CU28" s="44"/>
     </row>
-    <row r="29" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A29" s="58" t="s">
-        <v>30</v>
-      </c>
-      <c r="B29" s="33" t="s">
-        <v>32</v>
-      </c>
-      <c r="C29" s="75"/>
-      <c r="D29" s="34"/>
-      <c r="E29" s="35"/>
-      <c r="F29" s="36"/>
+    <row r="29" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1">
+      <c r="A29" s="58"/>
+      <c r="B29" s="81" t="s">
+        <v>29</v>
+      </c>
+      <c r="C29" s="76"/>
+      <c r="D29" s="37"/>
+      <c r="E29" s="67" t="s">
+        <v>39</v>
+      </c>
+      <c r="F29" s="67" t="s">
+        <v>39</v>
+      </c>
       <c r="G29" s="17"/>
-      <c r="H29" s="17" t="str">
-        <f t="shared" si="48"/>
-        <v/>
+      <c r="H29" s="17" t="e">
+        <f t="shared" ca="1" si="38"/>
+        <v>#VALUE!</v>
       </c>
       <c r="I29" s="44"/>
       <c r="J29" s="44"/>
@@ -4967,22 +4898,22 @@
       <c r="CT29" s="44"/>
       <c r="CU29" s="44"/>
     </row>
-    <row r="30" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A30" s="58"/>
       <c r="B30" s="81" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C30" s="76"/>
       <c r="D30" s="37"/>
       <c r="E30" s="67" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="F30" s="67" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="G30" s="17"/>
       <c r="H30" s="17" t="e">
-        <f>IF(OR(ISBLANK(task_start),ISBLANK(task_end)),"",task_end-task_start+1)</f>
+        <f t="shared" ca="1" si="38"/>
         <v>#VALUE!</v>
       </c>
       <c r="I30" s="44"/>
@@ -5077,22 +5008,22 @@
       <c r="CT30" s="44"/>
       <c r="CU30" s="44"/>
     </row>
-    <row r="31" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1">
       <c r="A31" s="58"/>
       <c r="B31" s="81" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C31" s="76"/>
       <c r="D31" s="37"/>
       <c r="E31" s="67" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="F31" s="67" t="s">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="G31" s="17"/>
       <c r="H31" s="17" t="e">
-        <f t="shared" si="48"/>
+        <f t="shared" ca="1" si="38"/>
         <v>#VALUE!</v>
       </c>
       <c r="I31" s="44"/>
@@ -5187,23 +5118,19 @@
       <c r="CT31" s="44"/>
       <c r="CU31" s="44"/>
     </row>
-    <row r="32" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A32" s="58"/>
-      <c r="B32" s="81" t="s">
-        <v>24</v>
-      </c>
-      <c r="C32" s="76"/>
-      <c r="D32" s="37"/>
-      <c r="E32" s="67" t="s">
-        <v>33</v>
-      </c>
-      <c r="F32" s="67" t="s">
-        <v>33</v>
-      </c>
+    <row r="32" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1">
+      <c r="A32" s="58" t="s">
+        <v>40</v>
+      </c>
+      <c r="B32" s="82"/>
+      <c r="C32" s="77"/>
+      <c r="D32" s="16"/>
+      <c r="E32" s="68"/>
+      <c r="F32" s="68"/>
       <c r="G32" s="17"/>
-      <c r="H32" s="17" t="e">
-        <f t="shared" si="48"/>
-        <v>#VALUE!</v>
+      <c r="H32" s="17" t="str">
+        <f t="shared" ca="1" si="38"/>
+        <v/>
       </c>
       <c r="I32" s="44"/>
       <c r="J32" s="44"/>
@@ -5297,449 +5224,123 @@
       <c r="CT32" s="44"/>
       <c r="CU32" s="44"/>
     </row>
-    <row r="33" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A33" s="58"/>
-      <c r="B33" s="81" t="s">
-        <v>25</v>
-      </c>
-      <c r="C33" s="76"/>
-      <c r="D33" s="37"/>
-      <c r="E33" s="67" t="s">
-        <v>33</v>
-      </c>
-      <c r="F33" s="67" t="s">
-        <v>33</v>
-      </c>
-      <c r="G33" s="17"/>
-      <c r="H33" s="17" t="e">
-        <f t="shared" si="48"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="I33" s="44"/>
-      <c r="J33" s="44"/>
-      <c r="K33" s="44"/>
-      <c r="L33" s="44"/>
-      <c r="M33" s="44"/>
-      <c r="N33" s="44"/>
-      <c r="O33" s="44"/>
-      <c r="P33" s="44"/>
-      <c r="Q33" s="44"/>
-      <c r="R33" s="44"/>
-      <c r="S33" s="44"/>
-      <c r="T33" s="44"/>
-      <c r="U33" s="44"/>
-      <c r="V33" s="44"/>
-      <c r="W33" s="44"/>
-      <c r="X33" s="44"/>
-      <c r="Y33" s="44"/>
-      <c r="Z33" s="44"/>
-      <c r="AA33" s="44"/>
-      <c r="AB33" s="44"/>
-      <c r="AC33" s="44"/>
-      <c r="AD33" s="44"/>
-      <c r="AE33" s="44"/>
-      <c r="AF33" s="44"/>
-      <c r="AG33" s="44"/>
-      <c r="AH33" s="44"/>
-      <c r="AI33" s="44"/>
-      <c r="AJ33" s="44"/>
-      <c r="AK33" s="44"/>
-      <c r="AL33" s="44"/>
-      <c r="AM33" s="44"/>
-      <c r="AN33" s="44"/>
-      <c r="AO33" s="44"/>
-      <c r="AP33" s="44"/>
-      <c r="AQ33" s="44"/>
-      <c r="AR33" s="44"/>
-      <c r="AS33" s="44"/>
-      <c r="AT33" s="44"/>
-      <c r="AU33" s="44"/>
-      <c r="AV33" s="44"/>
-      <c r="AW33" s="44"/>
-      <c r="AX33" s="44"/>
-      <c r="AY33" s="44"/>
-      <c r="AZ33" s="44"/>
-      <c r="BA33" s="44"/>
-      <c r="BB33" s="44"/>
-      <c r="BC33" s="44"/>
-      <c r="BD33" s="44"/>
-      <c r="BE33" s="44"/>
-      <c r="BF33" s="44"/>
-      <c r="BG33" s="44"/>
-      <c r="BH33" s="44"/>
-      <c r="BI33" s="44"/>
-      <c r="BJ33" s="44"/>
-      <c r="BK33" s="44"/>
-      <c r="BL33" s="44"/>
-      <c r="BM33" s="44"/>
-      <c r="BN33" s="44"/>
-      <c r="BO33" s="44"/>
-      <c r="BP33" s="44"/>
-      <c r="BQ33" s="44"/>
-      <c r="BR33" s="44"/>
-      <c r="BS33" s="44"/>
-      <c r="BT33" s="44"/>
-      <c r="BU33" s="44"/>
-      <c r="BV33" s="44"/>
-      <c r="BW33" s="44"/>
-      <c r="BX33" s="44"/>
-      <c r="BY33" s="44"/>
-      <c r="BZ33" s="44"/>
-      <c r="CA33" s="44"/>
-      <c r="CB33" s="44"/>
-      <c r="CC33" s="44"/>
-      <c r="CD33" s="44"/>
-      <c r="CE33" s="44"/>
-      <c r="CF33" s="44"/>
-      <c r="CG33" s="44"/>
-      <c r="CH33" s="44"/>
-      <c r="CI33" s="44"/>
-      <c r="CJ33" s="44"/>
-      <c r="CK33" s="44"/>
-      <c r="CL33" s="44"/>
-      <c r="CM33" s="44"/>
-      <c r="CN33" s="44"/>
-      <c r="CO33" s="44"/>
-      <c r="CP33" s="44"/>
-      <c r="CQ33" s="44"/>
-      <c r="CR33" s="44"/>
-      <c r="CS33" s="44"/>
-      <c r="CT33" s="44"/>
-      <c r="CU33" s="44"/>
+    <row r="33" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1">
+      <c r="A33" s="59" t="s">
+        <v>41</v>
+      </c>
+      <c r="B33" s="38" t="s">
+        <v>42</v>
+      </c>
+      <c r="C33" s="39"/>
+      <c r="D33" s="40"/>
+      <c r="E33" s="41"/>
+      <c r="F33" s="42"/>
+      <c r="G33" s="43"/>
+      <c r="H33" s="43" t="str">
+        <f t="shared" ca="1" si="38"/>
+        <v/>
+      </c>
+      <c r="I33" s="46"/>
+      <c r="J33" s="46"/>
+      <c r="K33" s="46"/>
+      <c r="L33" s="46"/>
+      <c r="M33" s="46"/>
+      <c r="N33" s="46"/>
+      <c r="O33" s="46"/>
+      <c r="P33" s="46"/>
+      <c r="Q33" s="46"/>
+      <c r="R33" s="46"/>
+      <c r="S33" s="46"/>
+      <c r="T33" s="46"/>
+      <c r="U33" s="46"/>
+      <c r="V33" s="46"/>
+      <c r="W33" s="46"/>
+      <c r="X33" s="46"/>
+      <c r="Y33" s="46"/>
+      <c r="Z33" s="46"/>
+      <c r="AA33" s="46"/>
+      <c r="AB33" s="46"/>
+      <c r="AC33" s="46"/>
+      <c r="AD33" s="46"/>
+      <c r="AE33" s="46"/>
+      <c r="AF33" s="46"/>
+      <c r="AG33" s="46"/>
+      <c r="AH33" s="46"/>
+      <c r="AI33" s="46"/>
+      <c r="AJ33" s="46"/>
+      <c r="AK33" s="46"/>
+      <c r="AL33" s="46"/>
+      <c r="AM33" s="46"/>
+      <c r="AN33" s="46"/>
+      <c r="AO33" s="46"/>
+      <c r="AP33" s="46"/>
+      <c r="AQ33" s="46"/>
+      <c r="AR33" s="46"/>
+      <c r="AS33" s="46"/>
+      <c r="AT33" s="46"/>
+      <c r="AU33" s="46"/>
+      <c r="AV33" s="46"/>
+      <c r="AW33" s="46"/>
+      <c r="AX33" s="46"/>
+      <c r="AY33" s="46"/>
+      <c r="AZ33" s="46"/>
+      <c r="BA33" s="46"/>
+      <c r="BB33" s="46"/>
+      <c r="BC33" s="46"/>
+      <c r="BD33" s="46"/>
+      <c r="BE33" s="46"/>
+      <c r="BF33" s="46"/>
+      <c r="BG33" s="46"/>
+      <c r="BH33" s="46"/>
+      <c r="BI33" s="46"/>
+      <c r="BJ33" s="46"/>
+      <c r="BK33" s="46"/>
+      <c r="BL33" s="46"/>
+      <c r="BM33" s="46"/>
+      <c r="BN33" s="46"/>
+      <c r="BO33" s="46"/>
+      <c r="BP33" s="46"/>
+      <c r="BQ33" s="46"/>
+      <c r="BR33" s="46"/>
+      <c r="BS33" s="46"/>
+      <c r="BT33" s="46"/>
+      <c r="BU33" s="46"/>
+      <c r="BV33" s="46"/>
+      <c r="BW33" s="46"/>
+      <c r="BX33" s="46"/>
+      <c r="BY33" s="46"/>
+      <c r="BZ33" s="46"/>
+      <c r="CA33" s="46"/>
+      <c r="CB33" s="46"/>
+      <c r="CC33" s="46"/>
+      <c r="CD33" s="46"/>
+      <c r="CE33" s="46"/>
+      <c r="CF33" s="46"/>
+      <c r="CG33" s="46"/>
+      <c r="CH33" s="46"/>
+      <c r="CI33" s="46"/>
+      <c r="CJ33" s="46"/>
+      <c r="CK33" s="46"/>
+      <c r="CL33" s="46"/>
+      <c r="CM33" s="46"/>
+      <c r="CN33" s="46"/>
+      <c r="CO33" s="46"/>
+      <c r="CP33" s="46"/>
+      <c r="CQ33" s="46"/>
+      <c r="CR33" s="46"/>
+      <c r="CS33" s="46"/>
+      <c r="CT33" s="46"/>
+      <c r="CU33" s="46"/>
     </row>
-    <row r="34" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A34" s="58"/>
-      <c r="B34" s="81" t="s">
-        <v>26</v>
-      </c>
-      <c r="C34" s="76"/>
-      <c r="D34" s="37"/>
-      <c r="E34" s="67" t="s">
-        <v>33</v>
-      </c>
-      <c r="F34" s="67" t="s">
-        <v>33</v>
-      </c>
-      <c r="G34" s="17"/>
-      <c r="H34" s="17" t="e">
-        <f t="shared" si="48"/>
-        <v>#VALUE!</v>
-      </c>
-      <c r="I34" s="44"/>
-      <c r="J34" s="44"/>
-      <c r="K34" s="44"/>
-      <c r="L34" s="44"/>
-      <c r="M34" s="44"/>
-      <c r="N34" s="44"/>
-      <c r="O34" s="44"/>
-      <c r="P34" s="44"/>
-      <c r="Q34" s="44"/>
-      <c r="R34" s="44"/>
-      <c r="S34" s="44"/>
-      <c r="T34" s="44"/>
-      <c r="U34" s="44"/>
-      <c r="V34" s="44"/>
-      <c r="W34" s="44"/>
-      <c r="X34" s="44"/>
-      <c r="Y34" s="44"/>
-      <c r="Z34" s="44"/>
-      <c r="AA34" s="44"/>
-      <c r="AB34" s="44"/>
-      <c r="AC34" s="44"/>
-      <c r="AD34" s="44"/>
-      <c r="AE34" s="44"/>
-      <c r="AF34" s="44"/>
-      <c r="AG34" s="44"/>
-      <c r="AH34" s="44"/>
-      <c r="AI34" s="44"/>
-      <c r="AJ34" s="44"/>
-      <c r="AK34" s="44"/>
-      <c r="AL34" s="44"/>
-      <c r="AM34" s="44"/>
-      <c r="AN34" s="44"/>
-      <c r="AO34" s="44"/>
-      <c r="AP34" s="44"/>
-      <c r="AQ34" s="44"/>
-      <c r="AR34" s="44"/>
-      <c r="AS34" s="44"/>
-      <c r="AT34" s="44"/>
-      <c r="AU34" s="44"/>
-      <c r="AV34" s="44"/>
-      <c r="AW34" s="44"/>
-      <c r="AX34" s="44"/>
-      <c r="AY34" s="44"/>
-      <c r="AZ34" s="44"/>
-      <c r="BA34" s="44"/>
-      <c r="BB34" s="44"/>
-      <c r="BC34" s="44"/>
-      <c r="BD34" s="44"/>
-      <c r="BE34" s="44"/>
-      <c r="BF34" s="44"/>
-      <c r="BG34" s="44"/>
-      <c r="BH34" s="44"/>
-      <c r="BI34" s="44"/>
-      <c r="BJ34" s="44"/>
-      <c r="BK34" s="44"/>
-      <c r="BL34" s="44"/>
-      <c r="BM34" s="44"/>
-      <c r="BN34" s="44"/>
-      <c r="BO34" s="44"/>
-      <c r="BP34" s="44"/>
-      <c r="BQ34" s="44"/>
-      <c r="BR34" s="44"/>
-      <c r="BS34" s="44"/>
-      <c r="BT34" s="44"/>
-      <c r="BU34" s="44"/>
-      <c r="BV34" s="44"/>
-      <c r="BW34" s="44"/>
-      <c r="BX34" s="44"/>
-      <c r="BY34" s="44"/>
-      <c r="BZ34" s="44"/>
-      <c r="CA34" s="44"/>
-      <c r="CB34" s="44"/>
-      <c r="CC34" s="44"/>
-      <c r="CD34" s="44"/>
-      <c r="CE34" s="44"/>
-      <c r="CF34" s="44"/>
-      <c r="CG34" s="44"/>
-      <c r="CH34" s="44"/>
-      <c r="CI34" s="44"/>
-      <c r="CJ34" s="44"/>
-      <c r="CK34" s="44"/>
-      <c r="CL34" s="44"/>
-      <c r="CM34" s="44"/>
-      <c r="CN34" s="44"/>
-      <c r="CO34" s="44"/>
-      <c r="CP34" s="44"/>
-      <c r="CQ34" s="44"/>
-      <c r="CR34" s="44"/>
-      <c r="CS34" s="44"/>
-      <c r="CT34" s="44"/>
-      <c r="CU34" s="44"/>
+    <row r="34" spans="1:99" ht="30" customHeight="1">
+      <c r="G34" s="6"/>
     </row>
-    <row r="35" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A35" s="58" t="s">
-        <v>34</v>
-      </c>
-      <c r="B35" s="82"/>
-      <c r="C35" s="77"/>
-      <c r="D35" s="16"/>
-      <c r="E35" s="68"/>
-      <c r="F35" s="68"/>
-      <c r="G35" s="17"/>
-      <c r="H35" s="17" t="str">
-        <f t="shared" si="48"/>
-        <v/>
-      </c>
-      <c r="I35" s="44"/>
-      <c r="J35" s="44"/>
-      <c r="K35" s="44"/>
-      <c r="L35" s="44"/>
-      <c r="M35" s="44"/>
-      <c r="N35" s="44"/>
-      <c r="O35" s="44"/>
-      <c r="P35" s="44"/>
-      <c r="Q35" s="44"/>
-      <c r="R35" s="44"/>
-      <c r="S35" s="44"/>
-      <c r="T35" s="44"/>
-      <c r="U35" s="44"/>
-      <c r="V35" s="44"/>
-      <c r="W35" s="44"/>
-      <c r="X35" s="44"/>
-      <c r="Y35" s="44"/>
-      <c r="Z35" s="44"/>
-      <c r="AA35" s="44"/>
-      <c r="AB35" s="44"/>
-      <c r="AC35" s="44"/>
-      <c r="AD35" s="44"/>
-      <c r="AE35" s="44"/>
-      <c r="AF35" s="44"/>
-      <c r="AG35" s="44"/>
-      <c r="AH35" s="44"/>
-      <c r="AI35" s="44"/>
-      <c r="AJ35" s="44"/>
-      <c r="AK35" s="44"/>
-      <c r="AL35" s="44"/>
-      <c r="AM35" s="44"/>
-      <c r="AN35" s="44"/>
-      <c r="AO35" s="44"/>
-      <c r="AP35" s="44"/>
-      <c r="AQ35" s="44"/>
-      <c r="AR35" s="44"/>
-      <c r="AS35" s="44"/>
-      <c r="AT35" s="44"/>
-      <c r="AU35" s="44"/>
-      <c r="AV35" s="44"/>
-      <c r="AW35" s="44"/>
-      <c r="AX35" s="44"/>
-      <c r="AY35" s="44"/>
-      <c r="AZ35" s="44"/>
-      <c r="BA35" s="44"/>
-      <c r="BB35" s="44"/>
-      <c r="BC35" s="44"/>
-      <c r="BD35" s="44"/>
-      <c r="BE35" s="44"/>
-      <c r="BF35" s="44"/>
-      <c r="BG35" s="44"/>
-      <c r="BH35" s="44"/>
-      <c r="BI35" s="44"/>
-      <c r="BJ35" s="44"/>
-      <c r="BK35" s="44"/>
-      <c r="BL35" s="44"/>
-      <c r="BM35" s="44"/>
-      <c r="BN35" s="44"/>
-      <c r="BO35" s="44"/>
-      <c r="BP35" s="44"/>
-      <c r="BQ35" s="44"/>
-      <c r="BR35" s="44"/>
-      <c r="BS35" s="44"/>
-      <c r="BT35" s="44"/>
-      <c r="BU35" s="44"/>
-      <c r="BV35" s="44"/>
-      <c r="BW35" s="44"/>
-      <c r="BX35" s="44"/>
-      <c r="BY35" s="44"/>
-      <c r="BZ35" s="44"/>
-      <c r="CA35" s="44"/>
-      <c r="CB35" s="44"/>
-      <c r="CC35" s="44"/>
-      <c r="CD35" s="44"/>
-      <c r="CE35" s="44"/>
-      <c r="CF35" s="44"/>
-      <c r="CG35" s="44"/>
-      <c r="CH35" s="44"/>
-      <c r="CI35" s="44"/>
-      <c r="CJ35" s="44"/>
-      <c r="CK35" s="44"/>
-      <c r="CL35" s="44"/>
-      <c r="CM35" s="44"/>
-      <c r="CN35" s="44"/>
-      <c r="CO35" s="44"/>
-      <c r="CP35" s="44"/>
-      <c r="CQ35" s="44"/>
-      <c r="CR35" s="44"/>
-      <c r="CS35" s="44"/>
-      <c r="CT35" s="44"/>
-      <c r="CU35" s="44"/>
+    <row r="35" spans="1:99" ht="30" customHeight="1">
+      <c r="C35" s="14"/>
+      <c r="F35" s="60"/>
     </row>
-    <row r="36" spans="1:99" s="3" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A36" s="59" t="s">
-        <v>35</v>
-      </c>
-      <c r="B36" s="38" t="s">
-        <v>36</v>
-      </c>
-      <c r="C36" s="39"/>
-      <c r="D36" s="40"/>
-      <c r="E36" s="41"/>
-      <c r="F36" s="42"/>
-      <c r="G36" s="43"/>
-      <c r="H36" s="43" t="str">
-        <f t="shared" si="48"/>
-        <v/>
-      </c>
-      <c r="I36" s="46"/>
-      <c r="J36" s="46"/>
-      <c r="K36" s="46"/>
-      <c r="L36" s="46"/>
-      <c r="M36" s="46"/>
-      <c r="N36" s="46"/>
-      <c r="O36" s="46"/>
-      <c r="P36" s="46"/>
-      <c r="Q36" s="46"/>
-      <c r="R36" s="46"/>
-      <c r="S36" s="46"/>
-      <c r="T36" s="46"/>
-      <c r="U36" s="46"/>
-      <c r="V36" s="46"/>
-      <c r="W36" s="46"/>
-      <c r="X36" s="46"/>
-      <c r="Y36" s="46"/>
-      <c r="Z36" s="46"/>
-      <c r="AA36" s="46"/>
-      <c r="AB36" s="46"/>
-      <c r="AC36" s="46"/>
-      <c r="AD36" s="46"/>
-      <c r="AE36" s="46"/>
-      <c r="AF36" s="46"/>
-      <c r="AG36" s="46"/>
-      <c r="AH36" s="46"/>
-      <c r="AI36" s="46"/>
-      <c r="AJ36" s="46"/>
-      <c r="AK36" s="46"/>
-      <c r="AL36" s="46"/>
-      <c r="AM36" s="46"/>
-      <c r="AN36" s="46"/>
-      <c r="AO36" s="46"/>
-      <c r="AP36" s="46"/>
-      <c r="AQ36" s="46"/>
-      <c r="AR36" s="46"/>
-      <c r="AS36" s="46"/>
-      <c r="AT36" s="46"/>
-      <c r="AU36" s="46"/>
-      <c r="AV36" s="46"/>
-      <c r="AW36" s="46"/>
-      <c r="AX36" s="46"/>
-      <c r="AY36" s="46"/>
-      <c r="AZ36" s="46"/>
-      <c r="BA36" s="46"/>
-      <c r="BB36" s="46"/>
-      <c r="BC36" s="46"/>
-      <c r="BD36" s="46"/>
-      <c r="BE36" s="46"/>
-      <c r="BF36" s="46"/>
-      <c r="BG36" s="46"/>
-      <c r="BH36" s="46"/>
-      <c r="BI36" s="46"/>
-      <c r="BJ36" s="46"/>
-      <c r="BK36" s="46"/>
-      <c r="BL36" s="46"/>
-      <c r="BM36" s="46"/>
-      <c r="BN36" s="46"/>
-      <c r="BO36" s="46"/>
-      <c r="BP36" s="46"/>
-      <c r="BQ36" s="46"/>
-      <c r="BR36" s="46"/>
-      <c r="BS36" s="46"/>
-      <c r="BT36" s="46"/>
-      <c r="BU36" s="46"/>
-      <c r="BV36" s="46"/>
-      <c r="BW36" s="46"/>
-      <c r="BX36" s="46"/>
-      <c r="BY36" s="46"/>
-      <c r="BZ36" s="46"/>
-      <c r="CA36" s="46"/>
-      <c r="CB36" s="46"/>
-      <c r="CC36" s="46"/>
-      <c r="CD36" s="46"/>
-      <c r="CE36" s="46"/>
-      <c r="CF36" s="46"/>
-      <c r="CG36" s="46"/>
-      <c r="CH36" s="46"/>
-      <c r="CI36" s="46"/>
-      <c r="CJ36" s="46"/>
-      <c r="CK36" s="46"/>
-      <c r="CL36" s="46"/>
-      <c r="CM36" s="46"/>
-      <c r="CN36" s="46"/>
-      <c r="CO36" s="46"/>
-      <c r="CP36" s="46"/>
-      <c r="CQ36" s="46"/>
-      <c r="CR36" s="46"/>
-      <c r="CS36" s="46"/>
-      <c r="CT36" s="46"/>
-      <c r="CU36" s="46"/>
-    </row>
-    <row r="37" spans="1:99" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="G37" s="6"/>
-    </row>
-    <row r="38" spans="1:99" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C38" s="14"/>
-      <c r="F38" s="60"/>
-    </row>
-    <row r="39" spans="1:99" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="C39" s="15"/>
+    <row r="36" spans="1:99" ht="30" customHeight="1">
+      <c r="C36" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="17">
@@ -5761,7 +5362,7 @@
     <mergeCell ref="CH4:CN4"/>
     <mergeCell ref="CO4:CU4"/>
   </mergeCells>
-  <conditionalFormatting sqref="D7:D36">
+  <conditionalFormatting sqref="D7:D33">
     <cfRule type="dataBar" priority="14">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -5775,12 +5376,12 @@
       </extLst>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I5:BL12 BM8:CU12 I13:CU36 CH5:CT5 BM5:CG6 CH6:CU6">
+  <conditionalFormatting sqref="I5:BL33 BM8:CU33 CH5:CT5 BM5:CG6 CH6:CU6">
     <cfRule type="expression" dxfId="3" priority="33">
       <formula>AND(TODAY()&gt;=I$5,TODAY()&lt;J$5)</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I7:BL12 BM8:CU12 I13:CU36">
+  <conditionalFormatting sqref="I7:BL33 BM8:CU33">
     <cfRule type="expression" dxfId="2" priority="27">
       <formula>AND(task_start&lt;=I$5,ROUNDDOWN((task_end-task_start+1)*task_progress,0)+task_start-1&gt;=I$5)</formula>
     </cfRule>
@@ -5805,7 +5406,7 @@
     <oddFooter>Page &amp;P of &amp;N</oddFooter>
   </headerFooter>
   <ignoredErrors>
-    <ignoredError sqref="F25:F26 E26" formula="1"/>
+    <ignoredError sqref="F22:F23 E23" formula="1"/>
   </ignoredErrors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
@@ -5823,7 +5424,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>D7:D36</xm:sqref>
+          <xm:sqref>D7:D33</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>
@@ -5834,88 +5435,88 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B16"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="13" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="14.1"/>
   <cols>
-    <col min="1" max="1" width="87.1796875" style="48" customWidth="1"/>
-    <col min="2" max="16384" width="9.1796875" style="2"/>
+    <col min="1" max="1" width="87.140625" style="48" customWidth="1"/>
+    <col min="2" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="46.5" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="1:2" s="50" customFormat="1" ht="15.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" ht="46.5" customHeight="1"/>
+    <row r="2" spans="1:2" s="50" customFormat="1" ht="15.95">
       <c r="A2" s="49" t="s">
-        <v>37</v>
+        <v>43</v>
       </c>
       <c r="B2" s="49"/>
     </row>
-    <row r="3" spans="1:2" s="54" customFormat="1" ht="27" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" s="54" customFormat="1" ht="27" customHeight="1">
       <c r="A3" s="55" t="s">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="B3" s="55"/>
     </row>
-    <row r="4" spans="1:2" s="51" customFormat="1" ht="26" x14ac:dyDescent="0.6">
+    <row r="4" spans="1:2" s="51" customFormat="1" ht="26.1">
       <c r="A4" s="52" t="s">
-        <v>39</v>
+        <v>45</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="74.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" ht="74.25" customHeight="1">
       <c r="A5" s="53" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" ht="26.25" customHeight="1">
       <c r="A6" s="52" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
     </row>
-    <row r="7" spans="1:2" s="48" customFormat="1" ht="205" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" s="48" customFormat="1" ht="204.95" customHeight="1">
       <c r="A7" s="57" t="s">
-        <v>42</v>
+        <v>48</v>
       </c>
     </row>
-    <row r="8" spans="1:2" s="51" customFormat="1" ht="26" x14ac:dyDescent="0.6">
+    <row r="8" spans="1:2" s="51" customFormat="1" ht="26.1">
       <c r="A8" s="52" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="58" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" ht="48">
       <c r="A9" s="53" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:2" s="48" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" s="48" customFormat="1" ht="27.95" customHeight="1">
       <c r="A10" s="56" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
     </row>
-    <row r="11" spans="1:2" s="51" customFormat="1" ht="26" x14ac:dyDescent="0.6">
+    <row r="11" spans="1:2" s="51" customFormat="1" ht="26.1">
       <c r="A11" s="52" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="29" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" ht="32.1">
       <c r="A12" s="53" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
     </row>
-    <row r="13" spans="1:2" s="48" customFormat="1" ht="28" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" s="48" customFormat="1" ht="27.95" customHeight="1">
       <c r="A13" s="56" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
     </row>
-    <row r="14" spans="1:2" s="51" customFormat="1" ht="26" x14ac:dyDescent="0.6">
+    <row r="14" spans="1:2" s="51" customFormat="1" ht="26.1">
       <c r="A14" s="52" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
     </row>
-    <row r="15" spans="1:2" ht="75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" ht="75" customHeight="1">
       <c r="A15" s="53" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
     </row>
-    <row r="16" spans="1:2" ht="72.5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" ht="63.95">
       <c r="A16" s="53" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>